<commit_message>
v0.4.9: The Phoenix Absolute Edition - Live Theme Customizer & Absolute Control UI
</commit_message>
<xml_diff>
--- a/data/destino_teste.xlsx
+++ b/data/destino_teste.xlsx
@@ -413,181 +413,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>CODIGO_EXTERNO</t>
+          <t>SAP_KEY</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>NOME_CLIENTE</t>
+          <t>SAP_VALOR</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>SALDO_CONTA</t>
+          <t>LIXO_1</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>DATA_CADASTRO</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>ATIVO</t>
+          <t>LIXO_2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Carlos Dias</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>150</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2023-01-01</t>
-        </is>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
+        <v>101</v>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dado inútil</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Daniela Souza</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2023-02-15</t>
-        </is>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
+        <v>102</v>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>888</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Eduardo Melo</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>300.5</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2023-03-10</t>
-        </is>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Helena Gomes</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>50</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2023-04-20</t>
-        </is>
-      </c>
-      <c r="E5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Igor Barros</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2023-05-05</t>
-        </is>
-      </c>
-      <c r="E6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Alice S.</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2022-10-10</t>
-        </is>
-      </c>
-      <c r="E7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Bruno C.</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>250</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2022-11-11</t>
-        </is>
-      </c>
-      <c r="E8" t="b">
-        <v>0</v>
+        <v>104</v>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>777</v>
       </c>
     </row>
   </sheetData>

</xml_diff>